<commit_message>
Export LMB : articles archivés présentés comme normaux (vitrine, recommande à la demande)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1wrBz23fxcbpQLqqeoHW8
</commit_message>
<xml_diff>
--- a/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
+++ b/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
@@ -72,7 +72,7 @@
     <t xml:space="preserve">- Colonne « Ancienne réf. (site) » : ce qui était renseigné sur PrestaShop, gardé pour mémoire. Les anciennes réf. sans « A- » ne sont pas des références LMB.</t>
   </si>
   <si>
-    <t xml:space="preserve">- Colonne « Article LMB » : Actif = article en vente dans LMB ; Archivé = article archivé dans LMB (souvent plus vendu en boutique). Un produit en ligne sur le site lié à un article archivé est à vérifier : le désactiver sur le site, ou le réactiver dans LMB.</t>
+    <t xml:space="preserve">- Colonne « Article LMB » : Actif = article en vente dans LMB ; Archivé = article archivé dans LMB. C'est normal pour des bouteilles rares gardées en vitrine et recommandées à la demande : la référence reste valable et le produit peut rester en vente sur le site.</t>
   </si>
   <si>
     <t xml:space="preserve">- Plusieurs produits du site partagent parfois la même réf. LMB : LMB regroupe certains parfums ou formats (ex. Nona 20 cl, Ginger &amp; Ginger, rhums arrangés 20 cl, places de dégustation).</t>
@@ -11800,7 +11800,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
         <v>15</v>
       </c>
@@ -13122,7 +13122,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>199</v>
       </c>
@@ -14698,7 +14698,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
         <v>383</v>
       </c>
@@ -16132,7 +16132,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
         <v>560</v>
       </c>
@@ -17694,7 +17694,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
         <v>745</v>
       </c>
@@ -18244,7 +18244,7 @@
         <v>806</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="7" t="s">
         <v>807</v>
       </c>
@@ -19736,7 +19736,7 @@
         <v>965</v>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="7" t="s">
         <v>966</v>
       </c>
@@ -20650,7 +20650,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
         <v>1052</v>
       </c>
@@ -20702,7 +20702,7 @@
         <v>1060</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="169.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
         <v>1052</v>
       </c>
@@ -22058,7 +22058,7 @@
         <v>1195</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="7" t="s">
         <v>1196</v>
       </c>
@@ -23268,7 +23268,7 @@
         <v>1312</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="7" t="s">
         <v>1313</v>
       </c>
@@ -24394,7 +24394,7 @@
         <v>1415</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="7" t="s">
         <v>1416</v>
       </c>
@@ -24498,7 +24498,7 @@
         <v>1425</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="7" t="s">
         <v>1426</v>
       </c>
@@ -26238,7 +26238,7 @@
         <v>1587</v>
       </c>
     </row>
-    <row r="264" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="264" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="7" t="s">
         <v>1588</v>
       </c>
@@ -26686,7 +26686,7 @@
         <v>1637</v>
       </c>
     </row>
-    <row r="272" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="7" t="s">
         <v>1638</v>
       </c>
@@ -38432,7 +38432,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="21" t="s">
         <v>554</v>
       </c>
@@ -38598,7 +38598,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="21" t="s">
         <v>622</v>
       </c>
@@ -38613,7 +38613,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="21" t="s">
         <v>628</v>
       </c>
@@ -38905,7 +38905,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="21" t="s">
         <v>745</v>
       </c>
@@ -38984,7 +38984,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="21" t="s">
         <v>775</v>
       </c>
@@ -39001,7 +39001,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="21" t="s">
         <v>782</v>
       </c>
@@ -39758,7 +39758,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="21" t="s">
         <v>1052</v>
       </c>
@@ -39773,7 +39773,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="21" t="s">
         <v>1052</v>
       </c>
@@ -40252,7 +40252,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="21" t="s">
         <v>1214</v>
       </c>
@@ -40363,7 +40363,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="21" t="s">
         <v>1252</v>
       </c>
@@ -40421,7 +40421,7 @@
         <v>422</v>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="21" t="s">
         <v>1271</v>
       </c>
@@ -40683,7 +40683,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="21" t="s">
         <v>1356</v>
       </c>
@@ -40713,7 +40713,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A218" s="21" t="s">
         <v>1366</v>
       </c>
@@ -40956,7 +40956,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="21" t="s">
         <v>1444</v>
       </c>
@@ -40971,7 +40971,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="21" t="s">
         <v>1449</v>
       </c>
@@ -41183,7 +41183,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="250" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A250" s="21"/>
       <c r="B250" s="21" t="s">
         <v>1517</v>
@@ -41348,7 +41348,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="261" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A261" s="21" t="s">
         <v>1571</v>
       </c>
@@ -41463,7 +41463,7 @@
         <v>504</v>
       </c>
     </row>
-    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="268" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A268" s="21" t="s">
         <v>1613</v>
       </c>
@@ -41480,7 +41480,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="269" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A269" s="21" t="s">
         <v>1620</v>
       </c>
@@ -41544,7 +41544,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="21" t="s">
         <v>1643</v>
       </c>
@@ -41724,7 +41724,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="285" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="21" t="s">
         <v>1700</v>
       </c>
@@ -41739,7 +41739,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="286" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A286" s="21" t="s">
         <v>1705</v>
       </c>
@@ -42251,7 +42251,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="318" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="21" t="s">
         <v>1877</v>
       </c>
@@ -42328,7 +42328,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="323" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A323" s="21" t="s">
         <v>1903</v>
       </c>
@@ -42388,7 +42388,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="327" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A327" s="21" t="s">
         <v>1919</v>
       </c>
@@ -42533,7 +42533,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="336" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="21" t="s">
         <v>1972</v>
       </c>
@@ -42601,7 +42601,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="340" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="21" t="s">
         <v>1993</v>
       </c>
@@ -42618,7 +42618,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="341" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="21" t="s">
         <v>1942</v>
       </c>
@@ -42635,7 +42635,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="342" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A342" s="21" t="s">
         <v>2001</v>
       </c>
@@ -42652,7 +42652,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="343" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="21" t="s">
         <v>2008</v>
       </c>
@@ -42686,7 +42686,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="345" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="21" t="s">
         <v>2022</v>
       </c>
@@ -42895,7 +42895,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="358" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="21" t="s">
         <v>2092</v>
       </c>
@@ -43141,7 +43141,7 @@
         <v>641</v>
       </c>
     </row>
-    <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="374" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A374" s="21" t="s">
         <v>2183</v>
       </c>
@@ -43307,7 +43307,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="384" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="21" t="s">
         <v>2236</v>
       </c>
@@ -43458,7 +43458,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="393" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="21" t="s">
         <v>2293</v>
       </c>
@@ -43526,7 +43526,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="397" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="21" t="s">
         <v>2318</v>
       </c>
@@ -43962,7 +43962,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="425" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="21" t="s">
         <v>2463</v>
       </c>
@@ -44274,7 +44274,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="445" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="21" t="s">
         <v>2573</v>
       </c>
@@ -44338,7 +44338,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="449" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="21" t="s">
         <v>2592</v>
       </c>
@@ -44540,7 +44540,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="461" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A461" s="21" t="s">
         <v>2641</v>
       </c>

</xml_diff>

<commit_message>
Site : 11 produits archivés désactivés (décision du patron), export LMB à jour
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1wrBz23fxcbpQLqqeoHW8
</commit_message>
<xml_diff>
--- a/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
+++ b/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
@@ -30,7 +30,7 @@
     <t xml:space="preserve">Export du catalogue PrestaShop (abcterroirs.com) avec les références LMB</t>
   </si>
   <si>
-    <t xml:space="preserve">Extrait le 16/10/2026 : 464 produits du site (344 actifs, 120 désactivés), rapprochés de l'extraction LMB « ETIQUETTES_PRIX_BD_au_141026 » puis vérifiés dans le catalogue LMB complet le 19/10/2026 (2 533 articles actifs + 4 725 archivés).</t>
+    <t xml:space="preserve">Extrait le 16/10/2026 : 464 produits du site (333 actifs, 131 désactivés), rapprochés de l'extraction LMB « ETIQUETTES_PRIX_BD_au_141026 » puis vérifiés dans le catalogue LMB complet le 19/10/2026 (2 533 articles actifs + 4 725 archivés).</t>
   </si>
   <si>
     <t xml:space="preserve">Colonne « Statut réf. LMB » (le décompte ci-dessous se met à jour tout seul) :</t>
@@ -2484,7 +2484,7 @@
     <t xml:space="preserve">GIN SAKURAO ORIGINAL - Japon</t>
   </si>
   <si>
-    <t xml:space="preserve">À ARCHIVER (décision du patron).</t>
+    <t xml:space="preserve">Archivé (décision du patron) : désactivé sur le site le 19/10/2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Gin Sakurao Original – Japon</t>
@@ -4882,7 +4882,7 @@
     <t xml:space="preserve">https://abcterroirs.com/index.php?id_product=481&amp;controller=product</t>
   </si>
   <si>
-    <t xml:space="preserve">À ARCHIVER (décision du patron). aucun « Triptyque » dans LMB</t>
+    <t xml:space="preserve">Archivé (décision du patron) : désactivé sur le site le 19/10/2026. aucun « Triptyque » dans LMB</t>
   </si>
   <si>
     <t xml:space="preserve">Triptyque – Distillerie Combier 20 cl</t>
@@ -5184,7 +5184,7 @@
     <t xml:space="preserve">BOITE DELICES ET GOURMANDISES sucrée salée Be happy Sweet Home</t>
   </si>
   <si>
-    <t xml:space="preserve">À ARCHIVER (décision du patron). LMB : boîte Délices et Gourmandises sucrée salée à 28,80 €</t>
+    <t xml:space="preserve">Archivé (décision du patron) : désactivé sur le site le 19/10/2026. LMB : boîte Délices et Gourmandises sucrée salée à 28,80 €</t>
   </si>
   <si>
     <t xml:space="preserve">Boîte Délices &amp; Gourmandises sucrée-salée</t>
@@ -17922,7 +17922,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
         <v>770</v>
       </c>
@@ -18081,7 +18081,7 @@
         <v>1.2</v>
       </c>
       <c r="Q110" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R110" s="10" t="n">
         <v>300</v>
@@ -18472,7 +18472,7 @@
         <v>831</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="7" t="s">
         <v>832</v>
       </c>
@@ -18746,7 +18746,7 @@
         <v>861</v>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="7" t="s">
         <v>862</v>
       </c>
@@ -19635,7 +19635,7 @@
         <v>1.5</v>
       </c>
       <c r="Q138" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R138" s="10" t="n">
         <v>348</v>
@@ -23284,7 +23284,7 @@
         <v>1315</v>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A207" s="7" t="s">
         <v>1316</v>
       </c>
@@ -24462,7 +24462,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="7" t="s">
         <v>1424</v>
       </c>
@@ -24817,7 +24817,7 @@
         <v>1.6</v>
       </c>
       <c r="Q236" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R236" s="10" t="n">
         <v>468</v>
@@ -24826,7 +24826,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="7" t="s">
         <v>1458</v>
       </c>
@@ -24984,7 +24984,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A240" s="7" t="s">
         <v>1476</v>
       </c>
@@ -25485,7 +25485,7 @@
         <v>1.27</v>
       </c>
       <c r="Q249" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R249" s="10" t="n">
         <v>482</v>
@@ -26256,7 +26256,7 @@
         <v>1591</v>
       </c>
     </row>
-    <row r="264" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="264" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A264" s="7" t="s">
         <v>1592</v>
       </c>
@@ -26411,7 +26411,7 @@
       <c r="O266" s="11"/>
       <c r="P266" s="10"/>
       <c r="Q266" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R266" s="10" t="n">
         <v>503</v>
@@ -26585,7 +26585,7 @@
         <v>1</v>
       </c>
       <c r="Q269" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R269" s="10" t="n">
         <v>508</v>
@@ -27289,7 +27289,7 @@
         <v>0.6</v>
       </c>
       <c r="Q282" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R282" s="10" t="n">
         <v>529</v>
@@ -27298,7 +27298,7 @@
         <v>1693</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="7" t="s">
         <v>1694</v>
       </c>
@@ -27399,7 +27399,7 @@
         <v>1.6</v>
       </c>
       <c r="Q284" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R284" s="10" t="n">
         <v>532</v>
@@ -27626,7 +27626,7 @@
         <v>1724</v>
       </c>
     </row>
-    <row r="289" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="289" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A289" s="7" t="s">
         <v>1715</v>
       </c>
@@ -29006,7 +29006,7 @@
         <v>1858</v>
       </c>
     </row>
-    <row r="314" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="314" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="7" t="s">
         <v>1859</v>
       </c>
@@ -29652,7 +29652,7 @@
         <v>1922</v>
       </c>
     </row>
-    <row r="326" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="326" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="7" t="s">
         <v>1923</v>
       </c>
@@ -30172,7 +30172,7 @@
         <v>1975</v>
       </c>
     </row>
-    <row r="336" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="336" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="7" t="s">
         <v>1976</v>
       </c>
@@ -31469,7 +31469,7 @@
         <v>1.4</v>
       </c>
       <c r="Q359" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R359" s="10" t="n">
         <v>622</v>
@@ -32721,7 +32721,7 @@
         <v>1.5</v>
       </c>
       <c r="Q382" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R382" s="10" t="n">
         <v>650</v>
@@ -33174,7 +33174,7 @@
         <v>2281</v>
       </c>
     </row>
-    <row r="391" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="391" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A391" s="15" t="s">
         <v>2282</v>
       </c>
@@ -34470,7 +34470,7 @@
         <v>2412</v>
       </c>
     </row>
-    <row r="415" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="415" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="7" t="s">
         <v>2413</v>
       </c>
@@ -35261,7 +35261,7 @@
       <c r="O429" s="11"/>
       <c r="P429" s="10"/>
       <c r="Q429" s="10" t="s">
-        <v>48</v>
+        <v>96</v>
       </c>
       <c r="R429" s="10" t="n">
         <v>711</v>
@@ -37314,7 +37314,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="21" t="s">
         <v>64</v>
       </c>
@@ -37429,7 +37429,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
         <v>118</v>
       </c>
@@ -37493,7 +37493,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="21" t="s">
         <v>149</v>
       </c>
@@ -37657,7 +37657,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
         <v>219</v>
       </c>
@@ -37706,7 +37706,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
         <v>238</v>
       </c>
@@ -37898,7 +37898,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="21" t="s">
         <v>314</v>
       </c>
@@ -38060,7 +38060,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="21" t="s">
         <v>384</v>
       </c>
@@ -38481,7 +38481,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="21" t="s">
         <v>561</v>
       </c>
@@ -38630,7 +38630,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="21" t="s">
         <v>623</v>
       </c>
@@ -38645,7 +38645,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="21" t="s">
         <v>630</v>
       </c>
@@ -38660,7 +38660,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="21" t="s">
         <v>636</v>
       </c>
@@ -38707,7 +38707,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="21" t="s">
         <v>656</v>
       </c>
@@ -38724,7 +38724,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="21" t="s">
         <v>662</v>
       </c>
@@ -38741,7 +38741,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="21" t="s">
         <v>668</v>
       </c>
@@ -38790,7 +38790,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="21" t="s">
         <v>687</v>
       </c>
@@ -38807,7 +38807,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="21" t="s">
         <v>694</v>
       </c>
@@ -38841,7 +38841,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="21" t="s">
         <v>706</v>
       </c>
@@ -38858,7 +38858,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="21" t="s">
         <v>713</v>
       </c>
@@ -38937,7 +38937,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="21" t="s">
         <v>747</v>
       </c>
@@ -38999,7 +38999,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="21" t="s">
         <v>770</v>
       </c>
@@ -39016,7 +39016,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="21" t="s">
         <v>777</v>
       </c>
@@ -39033,7 +39033,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="21" t="s">
         <v>784</v>
       </c>
@@ -39065,7 +39065,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="21" t="s">
         <v>798</v>
       </c>
@@ -39097,7 +39097,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="21" t="s">
         <v>810</v>
       </c>
@@ -39157,7 +39157,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="21" t="s">
         <v>832</v>
       </c>
@@ -39191,7 +39191,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="21" t="s">
         <v>843</v>
       </c>
@@ -39455,7 +39455,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="21" t="s">
         <v>939</v>
       </c>
@@ -39690,7 +39690,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="21" t="s">
         <v>1022</v>
       </c>
@@ -39707,7 +39707,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="21" t="s">
         <v>1029</v>
       </c>
@@ -39724,7 +39724,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="21" t="s">
         <v>1035</v>
       </c>
@@ -39758,7 +39758,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="21" t="s">
         <v>1044</v>
       </c>
@@ -39775,7 +39775,7 @@
         <v>368</v>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="21" t="s">
         <v>1048</v>
       </c>
@@ -39820,7 +39820,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="21" t="s">
         <v>1055</v>
       </c>
@@ -39850,7 +39850,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="21" t="s">
         <v>1048</v>
       </c>
@@ -39882,7 +39882,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="21" t="s">
         <v>1077</v>
       </c>
@@ -40065,7 +40065,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="21" t="s">
         <v>1137</v>
       </c>
@@ -40284,7 +40284,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="21" t="s">
         <v>1217</v>
       </c>
@@ -40844,7 +40844,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A225" s="21" t="s">
         <v>1401</v>
       </c>
@@ -40900,7 +40900,7 @@
         <v>459</v>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A229" s="21" t="s">
         <v>1419</v>
       </c>
@@ -40915,7 +40915,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="21" t="s">
         <v>1424</v>
       </c>
@@ -41018,7 +41018,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="21" t="s">
         <v>1458</v>
       </c>
@@ -41348,7 +41348,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="259" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A259" s="21" t="s">
         <v>1564</v>
       </c>
@@ -41446,7 +41446,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="265" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A265" s="21" t="s">
         <v>1597</v>
       </c>
@@ -41529,7 +41529,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="270" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A270" s="21" t="s">
         <v>1630</v>
       </c>
@@ -41546,7 +41546,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="271" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A271" s="21" t="s">
         <v>1637</v>
       </c>
@@ -41726,7 +41726,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="21" t="s">
         <v>1694</v>
       </c>
@@ -41741,7 +41741,7 @@
         <v>531</v>
       </c>
     </row>
-    <row r="284" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A284" s="21" t="s">
         <v>1699</v>
       </c>
@@ -41756,7 +41756,7 @@
         <v>532</v>
       </c>
     </row>
-    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A285" s="21" t="s">
         <v>1704</v>
       </c>
@@ -41801,7 +41801,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="288" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="21" t="s">
         <v>1715</v>
       </c>
@@ -41846,7 +41846,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="291" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A291" s="21" t="s">
         <v>1734</v>
       </c>
@@ -41861,7 +41861,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="292" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="21" t="s">
         <v>1739</v>
       </c>
@@ -41980,7 +41980,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="299" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A299" s="21" t="s">
         <v>1780</v>
       </c>
@@ -42089,7 +42089,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="306" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A306" s="21" t="s">
         <v>1819</v>
       </c>
@@ -42123,7 +42123,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="308" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="21" t="s">
         <v>1831</v>
       </c>
@@ -42187,7 +42187,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="312" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A312" s="21" t="s">
         <v>1847</v>
       </c>
@@ -42283,7 +42283,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="318" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A318" s="21" t="s">
         <v>1881</v>
       </c>
@@ -42315,7 +42315,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="320" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A320" s="21" t="s">
         <v>1892</v>
       </c>
@@ -42330,7 +42330,7 @@
         <v>575</v>
       </c>
     </row>
-    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="321" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A321" s="21" t="s">
         <v>1897</v>
       </c>
@@ -42375,7 +42375,7 @@
         <v>579</v>
       </c>
     </row>
-    <row r="324" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A324" s="21" t="s">
         <v>1912</v>
       </c>
@@ -42405,7 +42405,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="326" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A326" s="21" t="s">
         <v>1923</v>
       </c>
@@ -42420,7 +42420,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="327" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A327" s="21" t="s">
         <v>1923</v>
       </c>
@@ -42480,7 +42480,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="331" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="21" t="s">
         <v>1946</v>
       </c>
@@ -42531,7 +42531,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="334" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="21" t="s">
         <v>1965</v>
       </c>
@@ -42548,7 +42548,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="335" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A335" s="21" t="s">
         <v>1970</v>
       </c>
@@ -42565,7 +42565,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="336" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A336" s="21" t="s">
         <v>1976</v>
       </c>
@@ -42599,7 +42599,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="338" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A338" s="21" t="s">
         <v>1987</v>
       </c>
@@ -42616,7 +42616,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="339" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="21" t="s">
         <v>1992</v>
       </c>
@@ -42633,7 +42633,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="340" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="21" t="s">
         <v>1997</v>
       </c>
@@ -42650,7 +42650,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="341" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A341" s="21" t="s">
         <v>1946</v>
       </c>
@@ -42684,7 +42684,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="343" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A343" s="21" t="s">
         <v>2012</v>
       </c>
@@ -42701,7 +42701,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="344" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="21" t="s">
         <v>2020</v>
       </c>
@@ -42718,7 +42718,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="345" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A345" s="21" t="s">
         <v>2026</v>
       </c>
@@ -42752,7 +42752,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="347" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A347" s="21" t="s">
         <v>2038</v>
       </c>
@@ -42927,7 +42927,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="358" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A358" s="21" t="s">
         <v>2096</v>
       </c>
@@ -43034,7 +43034,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="365" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A365" s="21" t="s">
         <v>2135</v>
       </c>
@@ -43066,7 +43066,7 @@
         <v>633</v>
       </c>
     </row>
-    <row r="367" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A367" s="21" t="s">
         <v>2147</v>
       </c>
@@ -43141,7 +43141,7 @@
         <v>639</v>
       </c>
     </row>
-    <row r="372" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="21" t="s">
         <v>2175</v>
       </c>
@@ -43288,7 +43288,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="381" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="21" t="s">
         <v>2222</v>
       </c>
@@ -43339,7 +43339,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="384" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A384" s="21" t="s">
         <v>2240</v>
       </c>
@@ -43390,7 +43390,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="387" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="21" t="s">
         <v>2258</v>
       </c>
@@ -43424,7 +43424,7 @@
         <v>657</v>
       </c>
     </row>
-    <row r="389" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="21" t="s">
         <v>2271</v>
       </c>
@@ -43473,7 +43473,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="392" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="21" t="s">
         <v>2290</v>
       </c>
@@ -43558,7 +43558,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="397" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="21" t="s">
         <v>2322</v>
       </c>
@@ -43605,7 +43605,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="400" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A400" s="21" t="s">
         <v>2337</v>
       </c>
@@ -43761,7 +43761,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="410" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="21" t="s">
         <v>40</v>
       </c>
@@ -43778,7 +43778,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="411" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="21" t="s">
         <v>2391</v>
       </c>
@@ -43810,7 +43810,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="413" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A413" s="21" t="s">
         <v>2403</v>
       </c>
@@ -43825,7 +43825,7 @@
         <v>694</v>
       </c>
     </row>
-    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="414" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A414" s="21" t="s">
         <v>2408</v>
       </c>
@@ -43840,7 +43840,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="415" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="21" t="s">
         <v>2413</v>
       </c>
@@ -43855,7 +43855,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="416" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="21" t="s">
         <v>2418</v>
       </c>
@@ -43887,7 +43887,7 @@
         <v>698</v>
       </c>
     </row>
-    <row r="418" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="21" t="s">
         <v>2429</v>
       </c>
@@ -43994,7 +43994,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="425" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="21" t="s">
         <v>2466</v>
       </c>
@@ -44092,7 +44092,7 @@
         <v>712</v>
       </c>
     </row>
-    <row r="431" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A431" s="21" t="s">
         <v>2504</v>
       </c>
@@ -44107,7 +44107,7 @@
         <v>713</v>
       </c>
     </row>
-    <row r="432" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A432" s="21" t="s">
         <v>2509</v>
       </c>
@@ -44274,7 +44274,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="443" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A443" s="21" t="s">
         <v>2565</v>
       </c>
@@ -44306,7 +44306,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="445" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="21" t="s">
         <v>2576</v>
       </c>
@@ -44323,7 +44323,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="446" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="21" t="s">
         <v>2582</v>
       </c>

</xml_diff>

<commit_message>
Piq'Hans : 9 parfums supplémentaires (17 déclinaisons) avec leurs réfs LMB
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1wrBz23fxcbpQLqqeoHW8
</commit_message>
<xml_diff>
--- a/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
+++ b/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
@@ -7052,13 +7052,13 @@
     <t xml:space="preserve">https://abcterroirs.com/index.php?id_product=638&amp;controller=product</t>
   </si>
   <si>
-    <t xml:space="preserve">A-07148 / A-07154 / A-07147 / A-07157 / A-07150 / A-07153 / A-05658 / A-07159</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sauces Piq'Hans (8 parfums)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fiche passée en 8 déclinaisons « Parfum » le 19/10/2026, chaque parfum porte sa réf. LMB : L'Originale A-07148 · La Passionnée A-07154 · L'Atomique A-07147 · Deep Purple A-07157 · Taj Malave A-07150 · L'Enfumée A-07153 · Marble Queen A-05658 · Nectar Noir A-07159</t>
+    <t xml:space="preserve">A-07148 / A-07154 / A-07147 / A-07157 / A-07150 / A-07153 / A-05658 / A-07159 / A-07160 / A-07158 / A-07149 / A-07151 / A-07156 / A-07155 / A-07161 / A-07152 / A-07188</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sauces Piq'Hans (17 parfums)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiche passée en 17 déclinaisons « Parfum » le 19/10/2026, chaque parfum porte sa réf. LMB : L'Originale A-07148 · La Passionnée A-07154 · L'Atomique A-07147 · Deep Purple A-07157 · Taj Malave A-07150 · L'Enfumée A-07153 · Marble Queen A-05658 · Nectar Noir A-07159 · Caféinée A-07160 · Coco Rico A-07158 · Ensoleillé A-07149 · Jamaïcan Jerk A-07151 · Meyer A-07156 · Obsimo A-07155 · Pizza Yolo A-07161 · Waïpu A-07152 · Larme de Citrouille A-07188</t>
   </si>
   <si>
     <t xml:space="preserve">Sauces piquantes Piq'Hans – Nantes 10 cl</t>
@@ -16893,7 +16893,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
         <v>651</v>
       </c>
@@ -16949,7 +16949,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
         <v>659</v>
       </c>
@@ -18455,7 +18455,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="7" t="s">
         <v>829</v>
       </c>
@@ -19623,7 +19623,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="7" t="s">
         <v>954</v>
       </c>
@@ -19947,7 +19947,7 @@
         <v>986</v>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="7" t="s">
         <v>987</v>
       </c>
@@ -20649,7 +20649,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
         <v>1058</v>
       </c>
@@ -20701,7 +20701,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
         <v>1058</v>
       </c>
@@ -21565,7 +21565,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="7" t="s">
         <v>1140</v>
       </c>
@@ -22223,7 +22223,7 @@
         <v>1213</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="7" t="s">
         <v>1214</v>
       </c>
@@ -22333,7 +22333,7 @@
         <v>1225</v>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="7" t="s">
         <v>1226</v>
       </c>
@@ -24713,7 +24713,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="7" t="s">
         <v>1448</v>
       </c>
@@ -24873,7 +24873,7 @@
         <v>1463</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="7" t="s">
         <v>1464</v>
       </c>
@@ -25495,7 +25495,7 @@
         <v>1521</v>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A249" s="16"/>
       <c r="B249" s="8"/>
       <c r="C249" s="17" t="s">
@@ -26807,7 +26807,7 @@
         <v>1651</v>
       </c>
     </row>
-    <row r="273" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A273" s="7" t="s">
         <v>1652</v>
       </c>
@@ -27345,7 +27345,7 @@
         <v>1698</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="7" t="s">
         <v>1699</v>
       </c>
@@ -27617,7 +27617,7 @@
         <v>1726</v>
       </c>
     </row>
-    <row r="288" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="288" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="7" t="s">
         <v>1720</v>
       </c>
@@ -32125,7 +32125,7 @@
         <v>2174</v>
       </c>
     </row>
-    <row r="371" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="371" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A371" s="7" t="s">
         <v>2175</v>
       </c>
@@ -37460,7 +37460,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
         <v>105</v>
       </c>
@@ -37735,7 +37735,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
         <v>226</v>
       </c>
@@ -38663,7 +38663,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="21" t="s">
         <v>612</v>
       </c>
@@ -38710,7 +38710,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="21" t="s">
         <v>633</v>
       </c>
@@ -38872,7 +38872,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="21" t="s">
         <v>697</v>
       </c>
@@ -38889,7 +38889,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="21" t="s">
         <v>703</v>
       </c>
@@ -39207,7 +39207,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="21" t="s">
         <v>829</v>
       </c>
@@ -39454,7 +39454,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="21" t="s">
         <v>918</v>
       </c>
@@ -39520,7 +39520,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="21" t="s">
         <v>942</v>
       </c>
@@ -39537,7 +39537,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="21" t="s">
         <v>949</v>
       </c>
@@ -39569,7 +39569,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="21" t="s">
         <v>961</v>
       </c>
@@ -39738,7 +39738,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="21" t="s">
         <v>1018</v>
       </c>
@@ -39806,7 +39806,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="21" t="s">
         <v>1042</v>
       </c>
@@ -39885,7 +39885,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="21" t="s">
         <v>1058</v>
       </c>
@@ -39994,7 +39994,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="21" t="s">
         <v>1092</v>
       </c>
@@ -40130,7 +40130,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="21" t="s">
         <v>1140</v>
       </c>
@@ -40332,7 +40332,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="21" t="s">
         <v>1214</v>
       </c>
@@ -40349,7 +40349,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="21" t="s">
         <v>1220</v>
       </c>
@@ -40460,7 +40460,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="21" t="s">
         <v>1258</v>
       </c>
@@ -40475,7 +40475,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="21" t="s">
         <v>1263</v>
       </c>
@@ -40490,7 +40490,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="21" t="s">
         <v>1268</v>
       </c>
@@ -40707,7 +40707,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A211" s="21" t="s">
         <v>1339</v>
       </c>
@@ -40737,7 +40737,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="21" t="s">
         <v>1349</v>
       </c>
@@ -40780,7 +40780,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="21" t="s">
         <v>1362</v>
       </c>
@@ -40853,7 +40853,7 @@
         <v>449</v>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A221" s="21" t="s">
         <v>1386</v>
       </c>
@@ -40896,7 +40896,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="21" t="s">
         <v>1402</v>
       </c>
@@ -40926,7 +40926,7 @@
         <v>456</v>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A226" s="21" t="s">
         <v>1412</v>
       </c>
@@ -40982,7 +40982,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="21" t="s">
         <v>1430</v>
       </c>
@@ -40997,7 +40997,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="21" t="s">
         <v>1435</v>
       </c>
@@ -41040,7 +41040,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="21" t="s">
         <v>1448</v>
       </c>
@@ -41055,7 +41055,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A235" s="21" t="s">
         <v>1453</v>
       </c>
@@ -41070,7 +41070,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A236" s="21" t="s">
         <v>1458</v>
       </c>
@@ -41085,7 +41085,7 @@
         <v>468</v>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A237" s="21" t="s">
         <v>1464</v>
       </c>
@@ -41628,7 +41628,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="21" t="s">
         <v>1647</v>
       </c>
@@ -41793,7 +41793,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="21" t="s">
         <v>1699</v>
       </c>
@@ -41853,7 +41853,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="287" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A287" s="21" t="s">
         <v>1720</v>
       </c>
@@ -41979,7 +41979,7 @@
         <v>543</v>
       </c>
     </row>
-    <row r="295" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A295" s="21" t="s">
         <v>1761</v>
       </c>
@@ -42547,7 +42547,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="331" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="21" t="s">
         <v>1951</v>
       </c>
@@ -42598,7 +42598,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="334" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="21" t="s">
         <v>1970</v>
       </c>
@@ -42615,7 +42615,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="335" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A335" s="21" t="s">
         <v>1975</v>
       </c>
@@ -42649,7 +42649,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="337" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A337" s="21" t="s">
         <v>1986</v>
       </c>
@@ -43041,7 +43041,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="361" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="21" t="s">
         <v>2119</v>
       </c>
@@ -43357,7 +43357,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="381" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="21" t="s">
         <v>2230</v>
       </c>
@@ -43459,7 +43459,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="387" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="21" t="s">
         <v>2266</v>
       </c>
@@ -43559,7 +43559,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="393" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="21" t="s">
         <v>2305</v>
       </c>
@@ -43644,7 +43644,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="398" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="21" t="s">
         <v>2337</v>
       </c>
@@ -43779,7 +43779,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="407" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A407" s="21" t="s">
         <v>2381</v>
       </c>
@@ -44065,7 +44065,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="425" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="21" t="s">
         <v>2475</v>
       </c>
@@ -44298,7 +44298,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="440" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A440" s="21" t="s">
         <v>2558</v>
       </c>
@@ -44377,7 +44377,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="445" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A445" s="21" t="s">
         <v>2585</v>
       </c>
@@ -44394,7 +44394,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="446" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="21" t="s">
         <v>2591</v>
       </c>
@@ -44409,7 +44409,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="447" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A447" s="21" t="s">
         <v>2596</v>
       </c>
@@ -44441,7 +44441,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="449" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A449" s="21" t="s">
         <v>2604</v>
       </c>
@@ -44609,7 +44609,7 @@
         <v>745</v>
       </c>
     </row>
-    <row r="459" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A459" s="21" t="s">
         <v>2640</v>
       </c>
@@ -44643,7 +44643,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="461" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A461" s="21" t="s">
         <v>2652</v>
       </c>
@@ -44660,7 +44660,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="462" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A462" s="21" t="s">
         <v>2658</v>
       </c>
@@ -44711,7 +44711,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="465" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="21" t="s">
         <v>2673</v>
       </c>

</xml_diff>

<commit_message>
Piq'Hans : description avec les 17 parfums
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P1wrBz23fxcbpQLqqeoHW8
</commit_message>
<xml_diff>
--- a/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
+++ b/abc-terroirs/export-lmb/export-prestashop-pour-lmb.xlsx
@@ -7070,8 +7070,8 @@
 C'est pour cette raison que La Sauce Piqu'Hans s'est donnée une mission : proposer des sauces piquantes originales, goûteuses et à impact positif !</t>
   </si>
   <si>
-    <t xml:space="preserve">L'originale / La Passionnée / L'Atomique / Deep Purple / Taj Malave / L'enfumée / Marble Qeen / Nectar Noir et d'autres.
-N'hésitez pas nous contacter pour connaitre les disponibilités.</t>
+    <t xml:space="preserve">17 parfums au choix : L'Originale / La Passionnée / L'Atomique / Deep Purple / Taj Malave / L'Enfumée / Marble Queen / Nectar Noir / Caféinée / Coco Rico / Ensoleillé / Jamaïcan Jerk / Meyer / Obsimo / Pizza Yolo / Waïpu / Larme de Citrouille.
+Choisissez votre parfum dans la liste ci-dessus. N'hésitez pas à nous contacter pour connaître les disponibilités.</t>
   </si>
   <si>
     <t xml:space="preserve">Volume: 100ml</t>
@@ -10678,8 +10678,8 @@
 &lt;p&gt;C'est pour cette raison que La Sauce Piqu'Hans s'est donnée une mission : proposer des sauces piquantes originales, goûteuses et à impact positif !&lt;/p&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">&lt;p&gt;L'originale  /  La Passionnée   / L'Atomique   /  Deep Purple    /   Taj Malave   /  L'enfumée   /  Marble Qeen   /  Nectar Noir et d'autres.&lt;/p&gt;
-&lt;p&gt;N'hésitez pas nous contacter pour connaitre les disponibilités.&lt;/p&gt;</t>
+    <t xml:space="preserve">&lt;p&gt;17 parfums au choix : L'Originale / La Passionnée / L'Atomique / Deep Purple / Taj Malave / L'Enfumée / Marble Queen / Nectar Noir / Caféinée / Coco Rico / Ensoleillé / Jamaïcan Jerk / Meyer / Obsimo / Pizza Yolo / Waïpu / Larme de Citrouille.&lt;/p&gt;
+&lt;p&gt;Choisissez votre parfum dans la liste ci-dessus. N'hésitez pas à nous contacter pour connaître les disponibilités.&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;p&gt;Chaque sauce est pensée comme un voyage dans un flacon. Les recettes sont créées autour des origines historiques et géographiques des piments, pour reprendre des marqueurs gastronomiques phares de leurs terroirs.&lt;/p&gt;
@@ -13157,7 +13157,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
         <v>200</v>
       </c>
@@ -16949,7 +16949,7 @@
         <v>658</v>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
         <v>659</v>
       </c>
@@ -17741,7 +17741,7 @@
         <v>749</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
         <v>750</v>
       </c>
@@ -17795,7 +17795,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
         <v>756</v>
       </c>
@@ -17959,7 +17959,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
         <v>773</v>
       </c>
@@ -18293,7 +18293,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="7" t="s">
         <v>813</v>
       </c>
@@ -19623,7 +19623,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="7" t="s">
         <v>954</v>
       </c>
@@ -20649,7 +20649,7 @@
         <v>1057</v>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="7" t="s">
         <v>1058</v>
       </c>
@@ -20701,7 +20701,7 @@
         <v>1063</v>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="7" t="s">
         <v>1058</v>
       </c>
@@ -20753,7 +20753,7 @@
         <v>1066</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="147" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="7" t="s">
         <v>1058</v>
       </c>
@@ -21565,7 +21565,7 @@
         <v>1139</v>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="7" t="s">
         <v>1140</v>
       </c>
@@ -22111,7 +22111,7 @@
         <v>1201</v>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="7" t="s">
         <v>1202</v>
       </c>
@@ -27345,7 +27345,7 @@
         <v>1698</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="7" t="s">
         <v>1699</v>
       </c>
@@ -38710,7 +38710,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="21" t="s">
         <v>633</v>
       </c>
@@ -38906,7 +38906,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="21" t="s">
         <v>709</v>
       </c>
@@ -39017,7 +39017,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="21" t="s">
         <v>756</v>
       </c>
@@ -39130,7 +39130,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="21" t="s">
         <v>801</v>
       </c>
@@ -39738,7 +39738,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="21" t="s">
         <v>1018</v>
       </c>
@@ -39772,7 +39772,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="21" t="s">
         <v>1032</v>
       </c>
@@ -39806,7 +39806,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="21" t="s">
         <v>1042</v>
       </c>
@@ -39885,7 +39885,7 @@
         <v>373</v>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="21" t="s">
         <v>1058</v>
       </c>
@@ -39915,7 +39915,7 @@
         <v>375</v>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="21" t="s">
         <v>1051</v>
       </c>
@@ -39994,7 +39994,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="21" t="s">
         <v>1092</v>
       </c>
@@ -40332,7 +40332,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="21" t="s">
         <v>1214</v>
       </c>
@@ -40349,7 +40349,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="21" t="s">
         <v>1220</v>
       </c>
@@ -40460,7 +40460,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="21" t="s">
         <v>1258</v>
       </c>
@@ -40475,7 +40475,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="21" t="s">
         <v>1263</v>
       </c>
@@ -40490,7 +40490,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="21" t="s">
         <v>1268</v>
       </c>
@@ -40737,7 +40737,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A213" s="21" t="s">
         <v>1349</v>
       </c>
@@ -40780,7 +40780,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A216" s="21" t="s">
         <v>1362</v>
       </c>
@@ -40838,7 +40838,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A220" s="21" t="s">
         <v>1381</v>
       </c>
@@ -40896,7 +40896,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A224" s="21" t="s">
         <v>1402</v>
       </c>
@@ -40982,7 +40982,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A230" s="21" t="s">
         <v>1430</v>
       </c>
@@ -40997,7 +40997,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A231" s="21" t="s">
         <v>1435</v>
       </c>
@@ -41040,7 +41040,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A234" s="21" t="s">
         <v>1448</v>
       </c>
@@ -41481,7 +41481,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="263" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A263" s="21" t="s">
         <v>1591</v>
       </c>
@@ -41628,7 +41628,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="272" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A272" s="21" t="s">
         <v>1647</v>
       </c>
@@ -41793,7 +41793,7 @@
         <v>529</v>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A283" s="21" t="s">
         <v>1699</v>
       </c>
@@ -41868,7 +41868,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="288" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A288" s="21" t="s">
         <v>1720</v>
       </c>
@@ -41928,7 +41928,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A292" s="21" t="s">
         <v>1744</v>
       </c>
@@ -42288,7 +42288,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="314" customFormat="false" ht="124.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="21" t="s">
         <v>1864</v>
       </c>
@@ -42547,7 +42547,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="331" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A331" s="21" t="s">
         <v>1951</v>
       </c>
@@ -42598,7 +42598,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="334" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A334" s="21" t="s">
         <v>1970</v>
       </c>
@@ -42615,7 +42615,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="335" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A335" s="21" t="s">
         <v>1975</v>
       </c>
@@ -42683,7 +42683,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="339" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A339" s="21" t="s">
         <v>1997</v>
       </c>
@@ -42700,7 +42700,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="340" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A340" s="21" t="s">
         <v>2002</v>
       </c>
@@ -42768,7 +42768,7 @@
         <v>603</v>
       </c>
     </row>
-    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="344" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A344" s="21" t="s">
         <v>2025</v>
       </c>
@@ -43041,7 +43041,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="361" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A361" s="21" t="s">
         <v>2119</v>
       </c>
@@ -43357,7 +43357,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="381" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A381" s="21" t="s">
         <v>2230</v>
       </c>
@@ -43459,7 +43459,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="387" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A387" s="21" t="s">
         <v>2266</v>
       </c>
@@ -43559,7 +43559,7 @@
         <v>665</v>
       </c>
     </row>
-    <row r="393" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A393" s="21" t="s">
         <v>2305</v>
       </c>
@@ -43644,7 +43644,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="398" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="21" t="s">
         <v>2337</v>
       </c>
@@ -43796,7 +43796,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="408" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A408" s="21" t="s">
         <v>2387</v>
       </c>
@@ -44065,7 +44065,7 @@
         <v>706</v>
       </c>
     </row>
-    <row r="425" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A425" s="21" t="s">
         <v>2475</v>
       </c>
@@ -44394,7 +44394,7 @@
         <v>730</v>
       </c>
     </row>
-    <row r="446" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A446" s="21" t="s">
         <v>2591</v>
       </c>
@@ -44409,7 +44409,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="447" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A447" s="21" t="s">
         <v>2596</v>
       </c>
@@ -44711,7 +44711,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="465" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A465" s="21" t="s">
         <v>2673</v>
       </c>

</xml_diff>